<commit_message>
added speedup and maximum speedup for openmp
</commit_message>
<xml_diff>
--- a/metrics.xlsx
+++ b/metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9d064bda473745c9/Documenti/GitHub/High-Performance-Computing-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="750" documentId="8_{BF6E0229-5829-4C83-9BBC-58DCAFED2F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E47C8E0-EA36-4C42-8EDB-E54E5682ABCC}"/>
+  <xr:revisionPtr revIDLastSave="959" documentId="8_{BF6E0229-5829-4C83-9BBC-58DCAFED2F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFDB9A49-EFEF-4DF2-A4D4-9688882FAE76}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{674D654E-F57A-44BF-8654-EF23F1E7188E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{674D654E-F57A-44BF-8654-EF23F1E7188E}"/>
   </bookViews>
   <sheets>
     <sheet name="WK007" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="32">
   <si>
     <t>n</t>
   </si>
@@ -107,6 +107,36 @@
   <si>
     <t>precise</t>
   </si>
+  <si>
+    <t>Speed up</t>
+  </si>
+  <si>
+    <t>Maximum speedup n5000</t>
+  </si>
+  <si>
+    <t>MPI</t>
+  </si>
+  <si>
+    <t>CUDA</t>
+  </si>
+  <si>
+    <t>icx host precise standard</t>
+  </si>
+  <si>
+    <t>Maximum speedup n10000</t>
+  </si>
+  <si>
+    <t>Maximum speedup n15000</t>
+  </si>
+  <si>
+    <t>icc fast standard</t>
+  </si>
+  <si>
+    <t>icc fast fast-math standard</t>
+  </si>
+  <si>
+    <t>Speedup</t>
+  </si>
 </sst>
 </file>
 
@@ -121,12 +151,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -141,11 +177,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -480,16 +518,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7A0FC70-5187-461C-B4C6-97043A58D014}">
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:P105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="17.85546875" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="15.140625" customWidth="1"/>
     <col min="7" max="8" width="17.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" customWidth="1"/>
+    <col min="13" max="13" width="24.140625" customWidth="1"/>
+    <col min="14" max="14" width="11.28515625" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -514,25 +556,45 @@
       <c r="H1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>5000</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>5000</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="M2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2">
+        <f>MAX(I34:I57)</f>
+        <v>6.024096385542169</v>
+      </c>
+      <c r="P2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>5000</v>
       </c>
@@ -548,8 +610,11 @@
       <c r="E3">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5000</v>
       </c>
@@ -565,8 +630,11 @@
       <c r="E4">
         <v>256</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5000</v>
       </c>
@@ -583,7 +651,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5000</v>
       </c>
@@ -599,8 +667,21 @@
       <c r="E6">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" t="s">
+        <v>15</v>
+      </c>
+      <c r="O6">
+        <f>MAX(I58:I81)</f>
+        <v>8.4210526315789469</v>
+      </c>
+      <c r="P6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5000</v>
       </c>
@@ -616,8 +697,11 @@
       <c r="E7">
         <v>50</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5000</v>
       </c>
@@ -633,8 +717,11 @@
       <c r="E8">
         <v>6</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5000</v>
       </c>
@@ -651,7 +738,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>5000</v>
       </c>
@@ -667,8 +754,21 @@
       <c r="E10">
         <v>167</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="M10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" t="s">
+        <v>15</v>
+      </c>
+      <c r="O10">
+        <f>MAX(I82:I105)</f>
+        <v>8.778877887788779</v>
+      </c>
+      <c r="P10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5000</v>
       </c>
@@ -684,8 +784,11 @@
       <c r="E11">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>5000</v>
       </c>
@@ -701,8 +804,11 @@
       <c r="E12">
         <v>50</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>5000</v>
       </c>
@@ -719,24 +825,28 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>10000</v>
-      </c>
-      <c r="B14" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" t="s">
-        <v>6</v>
-      </c>
-      <c r="E14">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>10000</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E14" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>10000</v>
       </c>
@@ -753,7 +863,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10000</v>
       </c>
@@ -770,7 +880,7 @@
         <v>2066</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>10000</v>
       </c>
@@ -787,7 +897,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>10000</v>
       </c>
@@ -804,7 +914,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>10000</v>
       </c>
@@ -821,7 +931,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>10000</v>
       </c>
@@ -838,7 +948,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>10000</v>
       </c>
@@ -855,7 +965,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>10000</v>
       </c>
@@ -872,7 +982,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>10000</v>
       </c>
@@ -889,7 +999,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>10000</v>
       </c>
@@ -906,7 +1016,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>10000</v>
       </c>
@@ -923,7 +1033,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>15000</v>
       </c>
@@ -940,7 +1050,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>15000</v>
       </c>
@@ -957,7 +1067,7 @@
         <v>1313</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>15000</v>
       </c>
@@ -974,7 +1084,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>15000</v>
       </c>
@@ -991,24 +1101,28 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>15000</v>
-      </c>
-      <c r="B30" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" t="s">
-        <v>6</v>
-      </c>
-      <c r="E30">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>15000</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" s="2">
         <v>133</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>15000</v>
       </c>
@@ -1025,7 +1139,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>15000</v>
       </c>
@@ -1042,7 +1156,7 @@
         <v>1372</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>15000</v>
       </c>
@@ -1059,7 +1173,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5000</v>
       </c>
@@ -1078,8 +1192,12 @@
       <c r="G34" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I34">
+        <f>E2/E34</f>
+        <v>5.9523809523809526</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5000</v>
       </c>
@@ -1098,8 +1216,12 @@
       <c r="G35" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I35">
+        <f>E2/E35</f>
+        <v>2.3923444976076556</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5000</v>
       </c>
@@ -1118,8 +1240,12 @@
       <c r="G36" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I36">
+        <f>E2/E36</f>
+        <v>0.88495575221238931</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>5000</v>
       </c>
@@ -1138,8 +1264,12 @@
       <c r="G37" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I37">
+        <f>E2/E37</f>
+        <v>2.9239766081871346</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>5000</v>
       </c>
@@ -1158,8 +1288,12 @@
       <c r="G38" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I38">
+        <f>E2/E38</f>
+        <v>0.76103500761035003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>5000</v>
       </c>
@@ -1178,8 +1312,12 @@
       <c r="G39" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I39">
+        <f>E2/E39</f>
+        <v>2.2321428571428568</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>5000</v>
       </c>
@@ -1198,8 +1336,12 @@
       <c r="G40" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I40">
+        <f>E2/E40</f>
+        <v>0.7288629737609329</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>5000</v>
       </c>
@@ -1218,8 +1360,12 @@
       <c r="G41" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I41">
+        <f>E2/E41</f>
+        <v>2.3923444976076556</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>5000</v>
       </c>
@@ -1238,8 +1384,12 @@
       <c r="G42" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I42">
+        <f>E2/E42</f>
+        <v>5.6179775280898872</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>5000</v>
       </c>
@@ -1258,8 +1408,12 @@
       <c r="G43" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I43">
+        <f>E2/E43</f>
+        <v>3.7878787878787876</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>5000</v>
       </c>
@@ -1278,8 +1432,12 @@
       <c r="G44" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I44">
+        <f>E2/E44</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>5000</v>
       </c>
@@ -1298,8 +1456,12 @@
       <c r="G45" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I45">
+        <f>E2/E45</f>
+        <v>2.7027027027027026</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>5000</v>
       </c>
@@ -1318,8 +1480,12 @@
       <c r="G46" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I46">
+        <f>E2/E46</f>
+        <v>0.74294205052005935</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>5000</v>
       </c>
@@ -1338,8 +1504,12 @@
       <c r="G47" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I47">
+        <f>E2/E47</f>
+        <v>1.5625</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>5000</v>
       </c>
@@ -1358,8 +1528,12 @@
       <c r="G48" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I48">
+        <f>E2/E48</f>
+        <v>0.73313782991202348</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>5000</v>
       </c>
@@ -1378,8 +1552,12 @@
       <c r="G49" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I49">
+        <f>E2/E49</f>
+        <v>1.8050541516245486</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>5000</v>
       </c>
@@ -1401,8 +1579,12 @@
       <c r="G50" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I50">
+        <f>E2/E50</f>
+        <v>0.8771929824561403</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>5000</v>
       </c>
@@ -1424,8 +1606,12 @@
       <c r="G51" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I51">
+        <f>E2/E51</f>
+        <v>0.90744101633393837</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>5000</v>
       </c>
@@ -1447,8 +1633,12 @@
       <c r="G52" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I52">
+        <f>E2/E52</f>
+        <v>5.376344086021505</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>5000</v>
       </c>
@@ -1470,8 +1660,12 @@
       <c r="G53" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I53">
+        <f>E2/E53</f>
+        <v>6.024096385542169</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>5000</v>
       </c>
@@ -1493,8 +1687,12 @@
       <c r="G54" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I54">
+        <f>E2/E54</f>
+        <v>2.9069767441860463</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>5000</v>
       </c>
@@ -1516,8 +1714,12 @@
       <c r="G55" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I55">
+        <f>E2/E55</f>
+        <v>3.1055900621118009</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>5000</v>
       </c>
@@ -1539,8 +1741,12 @@
       <c r="G56" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I56">
+        <f>E2/E56</f>
+        <v>3.8759689922480618</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>5000</v>
       </c>
@@ -1562,8 +1768,12 @@
       <c r="G57" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I57">
+        <f>E2/E57</f>
+        <v>3.8461538461538458</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>10000</v>
       </c>
@@ -1582,8 +1792,12 @@
       <c r="G58" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I58">
+        <f>E14/E58</f>
+        <v>8.4210526315789469</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10000</v>
       </c>
@@ -1602,8 +1816,12 @@
       <c r="G59" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I59">
+        <f>E14/E59</f>
+        <v>2.7155465037338762</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>10000</v>
       </c>
@@ -1622,8 +1840,12 @@
       <c r="G60" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I60">
+        <f>E14/E60</f>
+        <v>0.82372322899505768</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10000</v>
       </c>
@@ -1642,8 +1864,12 @@
       <c r="G61" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I61">
+        <f>E14/E61</f>
+        <v>3.3898305084745761</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>10000</v>
       </c>
@@ -1662,8 +1888,12 @@
       <c r="G62" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I62">
+        <f>E14/E62</f>
+        <v>0.76628352490421447</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>10000</v>
       </c>
@@ -1682,8 +1912,12 @@
       <c r="G63" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I63">
+        <f>E14/E63</f>
+        <v>2.6863666890530555</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>10000</v>
       </c>
@@ -1702,8 +1936,12 @@
       <c r="G64" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I64">
+        <f>E14/E64</f>
+        <v>0.76452599388379205</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>10000</v>
       </c>
@@ -1722,8 +1960,12 @@
       <c r="G65" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I65">
+        <f>E14/E65</f>
+        <v>2.801120448179272</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>10000</v>
       </c>
@@ -1742,8 +1984,12 @@
       <c r="G66" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I66">
+        <f>E14/E66</f>
+        <v>6.3694267515923562</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>10000</v>
       </c>
@@ -1762,8 +2008,12 @@
       <c r="G67" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I67">
+        <f>E14/E67</f>
+        <v>4.5714285714285712</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>10000</v>
       </c>
@@ -1782,8 +2032,12 @@
       <c r="G68" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I68">
+        <f>E14/E68</f>
+        <v>5.9435364041604748</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>10000</v>
       </c>
@@ -1802,8 +2056,12 @@
       <c r="G69" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I69">
+        <f>E14/E69</f>
+        <v>3.3030553261767137</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>10000</v>
       </c>
@@ -1822,8 +2080,12 @@
       <c r="G70" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I70">
+        <f>E14/E70</f>
+        <v>0.71085836147147674</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>10000</v>
       </c>
@@ -1842,8 +2104,12 @@
       <c r="G71" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I71">
+        <f>E14/E71</f>
+        <v>2.0607934054611023</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>10000</v>
       </c>
@@ -1862,8 +2128,12 @@
       <c r="G72" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I72">
+        <f>E14/E72</f>
+        <v>0.72926162260711025</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>10000</v>
       </c>
@@ -1882,8 +2152,12 @@
       <c r="G73" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I73">
+        <f>E14/E73</f>
+        <v>1.733102253032929</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>10000</v>
       </c>
@@ -1905,8 +2179,12 @@
       <c r="G74" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I74">
+        <f>E14/E74</f>
+        <v>8.2815734989648035</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>10000</v>
       </c>
@@ -1928,8 +2206,12 @@
       <c r="G75" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I75">
+        <f>E14/E75</f>
+        <v>0.84033613445378152</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>10000</v>
       </c>
@@ -1951,8 +2233,12 @@
       <c r="G76" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I76">
+        <f>E14/E76</f>
+        <v>6.2208398133748055</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>10000</v>
       </c>
@@ -1974,8 +2260,12 @@
       <c r="G77" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I77">
+        <f>E14/E77</f>
+        <v>6.6445182724252501</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>10000</v>
       </c>
@@ -1997,8 +2287,12 @@
       <c r="G78" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I78">
+        <f>E14/E78</f>
+        <v>3.5087719298245612</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>10000</v>
       </c>
@@ -2020,8 +2314,12 @@
       <c r="G79" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I79">
+        <f>E14/E79</f>
+        <v>3.7037037037037033</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>10000</v>
       </c>
@@ -2043,8 +2341,12 @@
       <c r="G80" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I80">
+        <f>E14/E80</f>
+        <v>4.5300113250283127</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>10000</v>
       </c>
@@ -2066,8 +2368,12 @@
       <c r="G81" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I81">
+        <f>E14/E81</f>
+        <v>4.4843049327354256</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>15000</v>
       </c>
@@ -2086,8 +2392,12 @@
       <c r="G82" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I82">
+        <f>E30/E82</f>
+        <v>8.7730870712401057</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>15000</v>
       </c>
@@ -2106,8 +2416,12 @@
       <c r="G83" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I83">
+        <f>E30/E83</f>
+        <v>2.6906736799514466</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>15000</v>
       </c>
@@ -2126,8 +2440,12 @@
       <c r="G84" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I84">
+        <f>E30/E84</f>
+        <v>0.89901311342436119</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>15000</v>
       </c>
@@ -2146,8 +2464,12 @@
       <c r="G85" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I85">
+        <f>E30/E85</f>
+        <v>3.2510388658029825</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>15000</v>
       </c>
@@ -2166,8 +2488,12 @@
       <c r="G86" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I86">
+        <f>E30/E86</f>
+        <v>0.66436884959288678</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>15000</v>
       </c>
@@ -2186,8 +2512,12 @@
       <c r="G87" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I87">
+        <f>E30/E87</f>
+        <v>2.7220630372492836</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>15000</v>
       </c>
@@ -2206,8 +2536,12 @@
       <c r="G88" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I88">
+        <f>E30/E88</f>
+        <v>0.75757575757575757</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>15000</v>
       </c>
@@ -2226,8 +2560,12 @@
       <c r="G89" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I89">
+        <f>E30/E89</f>
+        <v>2.6798307475317347</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>15000</v>
       </c>
@@ -2246,8 +2584,12 @@
       <c r="G90" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I90">
+        <f>E30/E90</f>
+        <v>6.5906838453914771</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>15000</v>
       </c>
@@ -2266,8 +2608,12 @@
       <c r="G91" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I91">
+        <f>E30/E91</f>
+        <v>4.5407989074769546</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>15000</v>
       </c>
@@ -2286,8 +2632,12 @@
       <c r="G92" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I92">
+        <f>E30/E92</f>
+        <v>6.5324165029469548</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>15000</v>
       </c>
@@ -2306,8 +2656,12 @@
       <c r="G93" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I93">
+        <f>E30/E93</f>
+        <v>3.1704410011918949</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>15000</v>
       </c>
@@ -2326,8 +2680,12 @@
       <c r="G94" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I94">
+        <f>E30/E94</f>
+        <v>0.70684523809523814</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>15000</v>
       </c>
@@ -2346,8 +2704,12 @@
       <c r="G95" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I95">
+        <f>E30/E95</f>
+        <v>2.0729426433915212</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>15000</v>
       </c>
@@ -2366,8 +2728,12 @@
       <c r="G96" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I96">
+        <f>E30/E96</f>
+        <v>0.72610143582464381</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>15000</v>
       </c>
@@ -2386,8 +2752,12 @@
       <c r="G97" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I97">
+        <f>E30/E97</f>
+        <v>1.6538174583436955</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>15000</v>
       </c>
@@ -2409,8 +2779,12 @@
       <c r="G98" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I98">
+        <f>E30/E98</f>
+        <v>8.778877887788779</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>15000</v>
       </c>
@@ -2432,8 +2806,12 @@
       <c r="G99" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I99">
+        <f>E30/E99</f>
+        <v>0.88981066434736067</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>15000</v>
       </c>
@@ -2455,8 +2833,12 @@
       <c r="G100" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I100">
+        <f>E30/E100</f>
+        <v>6.8662880743417656</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>15000</v>
       </c>
@@ -2478,8 +2860,12 @@
       <c r="G101" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I101">
+        <f>E30/E101</f>
+        <v>6.7410035478966037</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>15000</v>
       </c>
@@ -2501,8 +2887,12 @@
       <c r="G102" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I102">
+        <f>E30/E102</f>
+        <v>3.3191914150237083</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>15000</v>
       </c>
@@ -2524,8 +2914,12 @@
       <c r="G103" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I103">
+        <f>E30/E103</f>
+        <v>2.6647966339410942</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>15000</v>
       </c>
@@ -2547,8 +2941,12 @@
       <c r="G104" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I104">
+        <f>E30/E104</f>
+        <v>4.4811320754716979</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>15000</v>
       </c>
@@ -2569,6 +2967,10 @@
       </c>
       <c r="G105" t="s">
         <v>18</v>
+      </c>
+      <c r="I105">
+        <f>E30/E105</f>
+        <v>4.4917257683215128</v>
       </c>
     </row>
   </sheetData>
@@ -2578,16 +2980,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A69E090-87CD-426F-B5E2-2BADFADD74B0}">
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="17.85546875" customWidth="1"/>
     <col min="4" max="4" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="15.140625" customWidth="1"/>
     <col min="7" max="8" width="17.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="13" max="13" width="26.140625" customWidth="1"/>
+    <col min="15" max="15" width="14.42578125" customWidth="1"/>
+    <col min="16" max="16" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2612,25 +3018,45 @@
       <c r="H1" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>5000</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>5000</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="M2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O2">
+        <f>MAX(I24:I39)</f>
+        <v>7.1428571428571432</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>5000</v>
       </c>
@@ -2646,8 +3072,11 @@
       <c r="E3">
         <v>257</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>5000</v>
       </c>
@@ -2663,8 +3092,11 @@
       <c r="E4">
         <v>68</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5000</v>
       </c>
@@ -2681,7 +3113,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5000</v>
       </c>
@@ -2697,25 +3129,44 @@
       <c r="E6">
         <v>48</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>5000</v>
-      </c>
-      <c r="B7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="M6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" t="s">
+        <v>15</v>
+      </c>
+      <c r="O6">
+        <f>MAX(I40:I63)</f>
+        <v>8.2987551867219906</v>
+      </c>
+      <c r="P6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>5000</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="3">
+        <v>5</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="N7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>5000</v>
       </c>
@@ -2731,8 +3182,11 @@
       <c r="E8">
         <v>167</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="N8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>5000</v>
       </c>
@@ -2749,7 +3203,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>5000</v>
       </c>
@@ -2765,8 +3219,21 @@
       <c r="E10">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="M10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N10" t="s">
+        <v>15</v>
+      </c>
+      <c r="O10">
+        <f>MAX(I64:I94)</f>
+        <v>9.1401489505754903</v>
+      </c>
+      <c r="P10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>5000</v>
       </c>
@@ -2782,25 +3249,35 @@
       <c r="E11">
         <v>49</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>10000</v>
-      </c>
-      <c r="B12" t="s">
-        <v>4</v>
-      </c>
-      <c r="C12" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E12">
+      <c r="N11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>10000</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="2">
         <v>40</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="N12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>10000</v>
       </c>
@@ -2817,7 +3294,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10000</v>
       </c>
@@ -2834,7 +3311,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>10000</v>
       </c>
@@ -2851,7 +3328,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>10000</v>
       </c>
@@ -2868,7 +3345,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>10000</v>
       </c>
@@ -2885,24 +3362,28 @@
         <v>407</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>15000</v>
-      </c>
-      <c r="B18" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" t="s">
-        <v>6</v>
-      </c>
-      <c r="E18">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>15000</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" s="2">
         <v>135</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>15000</v>
       </c>
@@ -2919,7 +3400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>15000</v>
       </c>
@@ -2936,7 +3417,7 @@
         <v>1365</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>15000</v>
       </c>
@@ -2953,7 +3434,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>15000</v>
       </c>
@@ -2970,7 +3451,7 @@
         <v>1358</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>15000</v>
       </c>
@@ -2987,7 +3468,7 @@
         <v>1374</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>5000</v>
       </c>
@@ -3006,8 +3487,12 @@
       <c r="G24" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I24">
+        <f>E2/E24</f>
+        <v>7.1428571428571432</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>5000</v>
       </c>
@@ -3026,8 +3511,12 @@
       <c r="G25" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I25">
+        <f>E2/E25</f>
+        <v>2.3148148148148149</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>5000</v>
       </c>
@@ -3046,8 +3535,12 @@
       <c r="G26" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I26">
+        <f>E2/E26</f>
+        <v>0.86058519793459554</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>5000</v>
       </c>
@@ -3066,8 +3559,12 @@
       <c r="G27" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I27">
+        <f>E2/E27</f>
+        <v>2.9069767441860463</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>5000</v>
       </c>
@@ -3086,8 +3583,12 @@
       <c r="G28" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I28">
+        <f>E2/E28</f>
+        <v>0.76452599388379205</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>5000</v>
       </c>
@@ -3106,8 +3607,12 @@
       <c r="G29" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I29">
+        <f>E2/E29</f>
+        <v>2.2727272727272725</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>5000</v>
       </c>
@@ -3126,8 +3631,12 @@
       <c r="G30" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I30">
+        <f>E2/E30</f>
+        <v>0.75528700906344415</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>5000</v>
       </c>
@@ -3146,8 +3655,12 @@
       <c r="G31" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I31">
+        <f>E2/E31</f>
+        <v>2.3809523809523809</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>5000</v>
       </c>
@@ -3166,8 +3679,12 @@
       <c r="G32" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I32">
+        <f>E2/E32</f>
+        <v>5.4347826086956523</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>5000</v>
       </c>
@@ -3186,8 +3703,12 @@
       <c r="G33" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I33">
+        <f>E2/E33</f>
+        <v>3.9370078740157481</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>5000</v>
       </c>
@@ -3206,8 +3727,12 @@
       <c r="G34" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I34">
+        <f>E2/E34</f>
+        <v>5.3191489361702127</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>5000</v>
       </c>
@@ -3226,8 +3751,12 @@
       <c r="G35" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I35">
+        <f>E2/E35</f>
+        <v>2.7173913043478262</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>5000</v>
       </c>
@@ -3246,8 +3775,12 @@
       <c r="G36" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I36">
+        <f>E2/E36</f>
+        <v>0.74738415545590431</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>5000</v>
       </c>
@@ -3266,8 +3799,12 @@
       <c r="G37" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I37">
+        <f>E2/E37</f>
+        <v>1.6233766233766234</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>5000</v>
       </c>
@@ -3286,8 +3823,12 @@
       <c r="G38" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I38">
+        <f>E2/E38</f>
+        <v>0.74850299401197606</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>5000</v>
       </c>
@@ -3306,8 +3847,12 @@
       <c r="G39" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I39">
+        <f>E2/E39</f>
+        <v>1.8518518518518516</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>10000</v>
       </c>
@@ -3326,8 +3871,12 @@
       <c r="G40" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I40">
+        <f>E12/E40</f>
+        <v>8.2135523613963031</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>10000</v>
       </c>
@@ -3346,8 +3895,12 @@
       <c r="G41" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I41">
+        <f>E12/E41</f>
+        <v>2.7303754266211602</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>10000</v>
       </c>
@@ -3366,8 +3919,12 @@
       <c r="G42" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I42">
+        <f>E12/E42</f>
+        <v>0.89405453732677687</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>10000</v>
       </c>
@@ -3386,8 +3943,12 @@
       <c r="G43" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I43">
+        <f>E12/E43</f>
+        <v>3.4393809114359413</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>10000</v>
       </c>
@@ -3406,8 +3967,12 @@
       <c r="G44" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I44">
+        <f>E12/E44</f>
+        <v>0.78201368523949166</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>10000</v>
       </c>
@@ -3426,8 +3991,12 @@
       <c r="G45" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I45">
+        <f>E12/E45</f>
+        <v>2.7643400138217</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>10000</v>
       </c>
@@ -3446,8 +4015,12 @@
       <c r="G46" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I46">
+        <f>E12/E46</f>
+        <v>0.76745970836531086</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>10000</v>
       </c>
@@ -3466,8 +4039,12 @@
       <c r="G47" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I47">
+        <f>E12/E47</f>
+        <v>2.6507620941020544</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>10000</v>
       </c>
@@ -3486,8 +4063,12 @@
       <c r="G48" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I48">
+        <f>E12/E48</f>
+        <v>6.5359477124183005</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>10000</v>
       </c>
@@ -3506,8 +4087,12 @@
       <c r="G49" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I49">
+        <f>E12/E49</f>
+        <v>4.489337822671156</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>10000</v>
       </c>
@@ -3526,8 +4111,12 @@
       <c r="G50" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I50">
+        <f>E12/E50</f>
+        <v>6.3492063492063497</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>10000</v>
       </c>
@@ -3546,8 +4135,12 @@
       <c r="G51" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I51">
+        <f>E12/E51</f>
+        <v>3.3333333333333335</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>10000</v>
       </c>
@@ -3566,8 +4159,12 @@
       <c r="G52" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I52">
+        <f>E12/E52</f>
+        <v>0.72293511657328757</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>10000</v>
       </c>
@@ -3586,8 +4183,12 @@
       <c r="G53" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I53">
+        <f>E12/E53</f>
+        <v>1.7436791630340016</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>10000</v>
       </c>
@@ -3606,8 +4207,12 @@
       <c r="G54" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I54">
+        <f>E12/E54</f>
+        <v>0.75301204819277112</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>10000</v>
       </c>
@@ -3626,8 +4231,12 @@
       <c r="G55" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I55">
+        <f>E12/E55</f>
+        <v>2.0703933747412009</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>10000</v>
       </c>
@@ -3649,8 +4258,12 @@
       <c r="G56" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I56">
+        <f>E12/E56</f>
+        <v>8.2987551867219906</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>10000</v>
       </c>
@@ -3672,8 +4285,12 @@
       <c r="G57" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I57">
+        <f>E12/E57</f>
+        <v>0.89485458612975388</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>10000</v>
       </c>
@@ -3695,8 +4312,12 @@
       <c r="G58" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I58">
+        <f>E12/E58</f>
+        <v>6.3795853269537481</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>10000</v>
       </c>
@@ -3718,8 +4339,12 @@
       <c r="G59" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I59">
+        <f>E12/E59</f>
+        <v>6.4620355411954762</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>10000</v>
       </c>
@@ -3741,8 +4366,12 @@
       <c r="G60" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I60">
+        <f>E12/E60</f>
+        <v>3.3528918692372174</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>10000</v>
       </c>
@@ -3764,8 +4393,12 @@
       <c r="G61" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I61">
+        <f>E12/E61</f>
+        <v>3.6630036630036629</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>10000</v>
       </c>
@@ -3787,8 +4420,12 @@
       <c r="G62" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I62">
+        <f>E12/E62</f>
+        <v>4.4296788482834994</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>10000</v>
       </c>
@@ -3810,8 +4447,12 @@
       <c r="G63" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I63">
+        <f>E12/E63</f>
+        <v>4.5351473922902494</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>15000</v>
       </c>
@@ -3830,8 +4471,12 @@
       <c r="G64" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I64">
+        <f>E18/E64</f>
+        <v>8.9641434262948199</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>15000</v>
       </c>
@@ -3850,8 +4495,12 @@
       <c r="G65" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I65">
+        <f>E18/E65</f>
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>15000</v>
       </c>
@@ -3870,8 +4519,12 @@
       <c r="G66" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I66">
+        <f>E18/E66</f>
+        <v>0.90835688332660469</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>15000</v>
       </c>
@@ -3890,8 +4543,12 @@
       <c r="G67" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I67">
+        <f>E18/E67</f>
+        <v>3.3267619517003451</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>15000</v>
       </c>
@@ -3910,8 +4567,12 @@
       <c r="G68" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I68">
+        <f>E18/E68</f>
+        <v>0.76348829317950462</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>15000</v>
       </c>
@@ -3930,8 +4591,12 @@
       <c r="G69" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I69">
+        <f>E18/E69</f>
+        <v>2.8043207312006646</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>15000</v>
       </c>
@@ -3950,8 +4615,12 @@
       <c r="G70" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I70">
+        <f>E18/E70</f>
+        <v>0.74458110418620038</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>15000</v>
       </c>
@@ -3970,8 +4639,12 @@
       <c r="G71" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I71">
+        <f>E18/E71</f>
+        <v>2.689243027888446</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>15000</v>
       </c>
@@ -3990,8 +4663,12 @@
       <c r="G72" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I72">
+        <f>E18/E72</f>
+        <v>7.0129870129870131</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>15000</v>
       </c>
@@ -4010,8 +4687,12 @@
       <c r="G73" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I73">
+        <f>E18/E73</f>
+        <v>4.6217048955837043</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>15000</v>
       </c>
@@ -4030,8 +4711,12 @@
       <c r="G74" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I74">
+        <f>E18/E74</f>
+        <v>6.8562722194007106</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>15000</v>
       </c>
@@ -4050,8 +4735,12 @@
       <c r="G75" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I75">
+        <f>E18/E75</f>
+        <v>3.2173498570066728</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>15000</v>
       </c>
@@ -4070,8 +4759,12 @@
       <c r="G76" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I76">
+        <f>E18/E76</f>
+        <v>0.7531380753138075</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>15000</v>
       </c>
@@ -4090,8 +4783,12 @@
       <c r="G77" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I77">
+        <f>E18/E77</f>
+        <v>2.0557332115121061</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>15000</v>
       </c>
@@ -4110,8 +4807,12 @@
       <c r="G78" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I78">
+        <f>E18/E78</f>
+        <v>0.74343300842557403</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>15000</v>
       </c>
@@ -4130,8 +4831,12 @@
       <c r="G79" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="I79">
+        <f>E18/E79</f>
+        <v>1.7136329017517136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>15000</v>
       </c>
@@ -4153,8 +4858,12 @@
       <c r="G80" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I80">
+        <f>E18/E80</f>
+        <v>9.1401489505754903</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>15000</v>
       </c>
@@ -4176,8 +4885,12 @@
       <c r="G81" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I81">
+        <f>E18/E81</f>
+        <v>0.90579710144927539</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>15000</v>
       </c>
@@ -4199,8 +4912,12 @@
       <c r="G82" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I82">
+        <f>E18/E82</f>
+        <v>6.7231075697211162</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>15000</v>
       </c>
@@ -4222,8 +4939,12 @@
       <c r="G83" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I83">
+        <f>E18/E83</f>
+        <v>6.743256743256743</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>15000</v>
       </c>
@@ -4245,8 +4966,12 @@
       <c r="G84" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I84">
+        <f>E18/E84</f>
+        <v>3.2545805207328837</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>15000</v>
       </c>
@@ -4268,8 +4993,12 @@
       <c r="G85" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I85">
+        <f>E18/E85</f>
+        <v>2.7444602561496239</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>15000</v>
       </c>
@@ -4291,8 +5020,12 @@
       <c r="G86" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I86">
+        <f>E18/E86</f>
+        <v>4.5747204337512706</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>15000</v>
       </c>
@@ -4314,8 +5047,12 @@
       <c r="G87" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I87">
+        <f>E18/E87</f>
+        <v>4.5577312626603641</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>15000</v>
       </c>
@@ -4337,8 +5074,12 @@
       <c r="H88">
         <v>1</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I88">
+        <f>E18/E88</f>
+        <v>0.99388942059927843</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>15000</v>
       </c>
@@ -4360,8 +5101,12 @@
       <c r="H89">
         <v>2</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I89">
+        <f>E18/E89</f>
+        <v>1.7921146953405018</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>15000</v>
       </c>
@@ -4383,8 +5128,12 @@
       <c r="H90">
         <v>4</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I90">
+        <f>E18/E90</f>
+        <v>3.8363171355498724</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>15000</v>
       </c>
@@ -4406,8 +5155,12 @@
       <c r="H91">
         <v>8</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I91">
+        <f>E18/E91</f>
+        <v>6.2586926286509037</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>15000</v>
       </c>
@@ -4429,8 +5182,12 @@
       <c r="H92">
         <v>16</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I92">
+        <f>E18/E92</f>
+        <v>7.8397212543554016</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>15000</v>
       </c>
@@ -4452,8 +5209,12 @@
       <c r="H93">
         <v>24</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I93">
+        <f>E18/E93</f>
+        <v>8.7662337662337659</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>15000</v>
       </c>
@@ -4474,6 +5235,10 @@
       </c>
       <c r="H94">
         <v>32</v>
+      </c>
+      <c r="I94">
+        <f>E18/E94</f>
+        <v>7.9834417504435242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>